<commit_message>
changed lf year variable to numeric; fixed saipe df to remove 2009 duplicates
</commit_message>
<xml_diff>
--- a/lf_data_2000_2010.xlsx
+++ b/lf_data_2000_2010.xlsx
@@ -367,7 +367,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>County FIPS Code</t>
+          <t>fips_county</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -377,7 +377,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>year</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>